<commit_message>
New MYSQL scripts added
</commit_message>
<xml_diff>
--- a/Excel/index match.xlsx
+++ b/Excel/index match.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Abror All Materials\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Arbor all Folder\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2336044-1B0E-41FA-B439-427D466F9807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369A02D5-B8AC-43BD-8B43-0E31C1C5E59E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1FEF1213-5C6B-40E1-9D8B-A47D6B5A2DBE}"/>
   </bookViews>
@@ -682,7 +682,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -693,6 +693,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -758,7 +766,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -785,6 +793,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1106,7 +1117,7 @@
   <cols>
     <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.5546875" customWidth="1"/>
+    <col min="11" max="11" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -1892,13 +1903,13 @@
         <v>57</v>
       </c>
     </row>
-    <row r="56" spans="9:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="9:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="J56" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="K56" s="9" t="e">
-        <f>INDEX(C2:G21,MATCH(J55,B2:B21,0),MATCH(K55,C1:G1,0))</f>
-        <v>#N/A</v>
+      <c r="K56" s="10" t="str">
+        <f>IFERROR(INDEX(C2:G21,MATCH(J55,B2:B21,0),MATCH(K55,C1:G1,0)),"Subject Not Found")</f>
+        <v>Subject Not Found</v>
       </c>
     </row>
     <row r="57" spans="9:11" x14ac:dyDescent="0.3">

</xml_diff>